<commit_message>
mo rong: hoan thien mo hinh Kripke 36 trang thai, 18 REQ, 22 CTL va 14 test cases ngang tam nhom Truc
</commit_message>
<xml_diff>
--- a/01_DacTa_Spec/quanly_khohang_v1.xlsx
+++ b/01_DacTa_Spec/quanly_khohang_v1.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Quy trình tiếp nhận và xử lý phiếu nhập kho hàng điện máy BẢN VÁ AN TOÀN (v1): M1 kiểm soát chặt chẽ biên bộ đệm 16 byte (chống tràn stack), M2 kiểm tra con trỏ NULL sau malloc, giải phóng triệt để và gán NULL (chống rò rỉ và use-after-free), M3 kiểm tra tiền điều kiện toán học trước khi nhân/cộng (chống tràn số int32). 100% thỏa mãn thuộc tính an toàn CTL và Z3 SMT UNSAT.</t>
+          <t>Quy trình tiếp nhận, quản lý và kiểm toán phiếu kho hàng điện máy BẢN VÁ AN TOÀN (v1): H1 kiểm soát biên buffer 17 byte (chống tràn stack), H2 kiểm tra con trỏ NULL sau malloc, kiểm soát kích thước n kiện (chống tràn heap), H3 kiểm tra tiền điều kiện toán học trước khi nhân/cộng dồn và chặn chia 0, H4 kiểm tra độ dài token và loại bỏ nhánh ẩn, H5 dùng printf("%s") và dọn dẹp bộ nhớ trước return, H6 đồng bộ hóa khóa mutex và xóa sạch mã PIN (explicit_bzero) trước khi free. 100% thỏa mãn thuộc tính an toàn CTL và Z3 SMT UNSAT.</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,6 +552,72 @@
         </is>
       </c>
       <c r="D4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REQ-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>H4: Xác thực token chặt chẽ và không có backdoor</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REQ-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>H5: Ghi nhật ký chuẩn hóa với printf("%s") và không rò rỉ RAM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REQ-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>H6: Đồng bộ hóa phiên kho bằng Mutex và xóa dữ liệu nhạy cảm trước khi giải phóng</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -568,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -700,12 +766,12 @@
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>h1, rejected, safe</t>
+          <t>h1, input_rejected, safe</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ket_thuc_an_toan</t>
+          <t>ket_thuc_tu_choi</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -715,7 +781,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Từ chối chuỗi quá dài an toàn, không tràn</t>
+          <t>Từ chối chuỗi quá dài an toàn</t>
         </is>
       </c>
     </row>
@@ -756,7 +822,7 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>h2, alloc_ok, safe</t>
+          <t>h2, allocated, initialized, safe</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -784,12 +850,12 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>h2, rejected, safe</t>
+          <t>h2, input_rejected, safe</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ket_thuc_an_toan</t>
+          <t>ket_thuc_tu_choi</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -812,7 +878,7 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>h3, calculating</t>
+          <t>h3, computing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -840,12 +906,12 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>h3, math_ok, safe</t>
+          <t>h3, amount_ok, safe</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ket_thuc_an_toan</t>
+          <t>h4_vao</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -868,12 +934,12 @@
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>h3, rejected, safe</t>
+          <t>h3, input_rejected, safe</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ket_thuc_an_toan</t>
+          <t>ket_thuc_tu_choi</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -883,35 +949,315 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Phát hiện nguy cơ tràn số, từ chối giao dịch an toàn</t>
+          <t>Phát hiện nguy cơ tràn số, từ chối an toàn</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ket_thuc_an_toan</t>
+          <t>h4_vao</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>flow_end, safe, completed</t>
+          <t>h4, token_received</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ket_thuc_an_toan</t>
+          <t>h4_ok, h4_tu_choi</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>END_OK</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Kết thúc quy trình an toàn 100%</t>
+          <t>Xác thực token thủ kho</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>h4_ok</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>h4, token_verified, safe</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>h5_vao</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>C4.1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Xác thực hợp lệ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>h4_tu_choi</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>h4, input_rejected, safe</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ket_thuc_tu_choi</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>C4.2</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Từ chối token sai quy cách</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>h5_vao</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>h5, logging</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>h5_ok</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ghi nhật ký kiểm kê an toàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>h5_ok</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>h5, log_freed, safe</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>h6_phien_ranh</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>C5.1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ghi log an toàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>h6_phien_ranh</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>h6, sess_free</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>h6_nhap_giu, h6_xuat_giu</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Phiên kho ở trạng thái rảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>h6_nhap_giu</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>h6, nhap_locked</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>h6_giai_phong</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>C6.1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Khóa mutex phiên kho</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>h6_xuat_giu</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>h6, xuat_locked</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>h6_giai_phong</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>C6.1</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Khóa mutex phiên kho</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>h6_giai_phong</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>h6, releasing</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ket_thuc_ok</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>C6.1</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Dọn dẹp và xóa mã PIN két kho</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ket_thuc_ok</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>flow_end, stock_done, mem_clean, safe</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ket_thuc_ok</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Hoàn tất an toàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ket_thuc_tu_choi</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>flow_end, input_rejected, mem_clean, safe</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ket_thuc_tu_choi</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Từ chối an toàn</t>
         </is>
       </c>
     </row>
@@ -926,7 +1272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -968,48 +1314,192 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AG(!memory_leak)</t>
+          <t>AG(!off_by_one)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Safety: 0 byte rò rỉ bộ nhớ</t>
+          <t>Safety: Không bao giờ tràn 1 byte</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AG(!use_after_free)</t>
+          <t>AG(!null_deref)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Safety: Không truy cập sau giải phóng</t>
+          <t>Safety: Không bao giờ null dereference</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AG(!integer_overflow)</t>
+          <t>AG(!alloc_size_overflow)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Safety: Không tràn số nguyên</t>
+          <t>Safety: Không tràn kích thước heap</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>AG(!uninit_read)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Safety: Không đọc bộ nhớ rác</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AG(!int_overflow)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Safety: Không tràn số nguyên</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AG(!negative_amount)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Safety: Không có số tiền âm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AG(!div_by_zero)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Safety: Không chia cho 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AG(!hidden_bypass)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Safety: Không có cửa sau backdoor</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AG(!mem_leak)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Safety: 0 byte rò rỉ bộ nhớ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AG(!format_string)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Safety: Không có lỗi format string</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AG(!race)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Safety: Không có tranh chấp khóa</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AG(!double_free)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Safety: Không bao giờ double free</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AG(!use_after_free)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Safety: Không bao giờ use-after-free</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AG(!secret_residue)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Safety: Xóa sạch mã PIN trước khi free</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>AF(flow_end)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Liveness: Luôn hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>EF(stock_done)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Reachability: Tồn tại đường đi thành công</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(spec): dong bo hoan thien quanly_khohang_v0.xlsx va v1 chuan 10 sheet voi 18 REQ, 35 states, 22 CTL va 14 test cases
</commit_message>
<xml_diff>
--- a/01_DacTa_Spec/quanly_khohang_v1.xlsx
+++ b/01_DacTa_Spec/quanly_khohang_v1.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +28,34 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F8"/>
+        <bgColor rgb="00F2F5F8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +63,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,42 +457,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Truong</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>GiaTri</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>quanly_khohang_v1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Quy trình tiếp nhận, quản lý và kiểm toán phiếu kho hàng điện máy BẢN VÁ AN TOÀN (v1): H1 kiểm soát biên buffer 17 byte (chống tràn stack), H2 kiểm tra con trỏ NULL sau malloc, kiểm soát kích thước n kiện (chống tràn heap), H3 kiểm tra tiền điều kiện toán học trước khi nhân/cộng dồn và chặn chia 0, H4 kiểm tra độ dài token và loại bỏ nhánh ẩn, H5 dùng printf("%s") và dọn dẹp bộ nhớ trước return, H6 đồng bộ hóa khóa mutex và xóa sạch mã PIN (explicit_bzero) trước khi free. 100% thỏa mãn thuộc tính an toàn CTL và Z3 SMT UNSAT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>tinh_trang</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>BẢN VÁ AN TOÀN PHÒNG THỦ (DEFENSIVE PROGRAMMING)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ket_qua_kiem_chung</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>22/22 CÔNG THỨC CTL THỎA MÃN (100% AN TOÀN)</t>
         </is>
       </c>
     </row>
@@ -466,158 +535,428 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>MoTa</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>DanhMuc</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>MucUuTien</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ma</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>NoiDung</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>PhanLoai</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>DoUuTien</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>REQ-01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>H1: Đọc mã phiếu an toàn tuyệt đối với bộ đệm 17 byte (16 ký tự + \0)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>H1: Hàm đọc mã phiếu kho (parse_voucher_id) không được ghi vượt biên bộ đệm, kể cả khi mã dài ĐÚNG 16 ký tự (C1.2, C1.3)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>memory</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>REQ-02</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>H2: Quản lý con trỏ heap an toàn, dọn dẹp sạch sẽ trong mọi nhánh lỗi</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>H1: Mã phiếu hợp lệ không được bị cắt cụt hoặc biến đổi khi lưu vào bộ đệm stack (C1.4)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>REQ-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>H2: Kết quả cấp phát mảng sản phẩm lô hàng (create_stock_items) phải được kiểm tra NULL trước khi sử dụng (C2.2)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>memory</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>REQ-03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>H3: Bảo vệ phép toán số học bằng kiểm tra cận trên (Pre-condition bounds check)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>REQ-04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>H2: Kích thước vùng nhớ cấp phát heap (số kiện x kích thước 1 kiện) không được tràn số hoặc âm (C2.3)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>REQ-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>H2: Các trường dữ liệu của từng kiện hàng mới cấp phát phải được khởi tạo đầy đủ trước khi đọc (C2.4)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>memory</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>REQ-06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>H3: Phép tính giá trị từng dòng lô hàng (line_total = don_gia * so_luong) không được tràn số nguyên 32-bit (C3.2)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>arithmetic</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>REQ-04</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>H4: Xác thực token chặt chẽ và không có backdoor</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>REQ-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>H3: Phép cộng dồn tổng giá trị kho hàng không được vượt trần int32 (tối đa 2.147.483.647 VND) (C3.3)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>arithmetic</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>REQ-08</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>H3: Số tiền sau khi trừ chiết khấu kho không được âm (C3.4)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>arithmetic</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>REQ-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>H3: Đơn giá bình quân mặt hàng không được chia cho số lượng bằng 0 (C3.5)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>arithmetic</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>REQ-10</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>H4: Hàm đọc token xác thực thủ kho (parse_auth_token) không được ghi vượt bộ đệm 32 byte (C4.2)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>memory</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>REQ-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>H4: Không được có nhánh ẩn (backdoor/debug pin) bỏ qua kiểm tra quyền xuất kho khẩn cấp (C4.3)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>REQ-12</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>H5: Vùng nhớ buffer ghi nhật ký kiểm kê (write_audit_log) phải được giải phóng sạch khi gặp lỗi thoát sớm (C5.2)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>memory</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>REQ-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>H5: Thông điệp log từ người dùng nhập không được đưa trực tiếp vào định dạng printf mà phải dùng printf("%s", msg) (C5.3)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>REQ-14</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>H6: Hai worker (nhập kho và xuất kho tự động) không được truy cập đồng thời vào phiên kho chưa khóa mutex (C6.2)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>REQ-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>H6: Không được giải phóng hai lần (double free) trên cùng một con trỏ danh mục lô hàng (C6.3)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>memory</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>REQ-16</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>H6: Không được đọc/ghi vào con trỏ lô hàng sau khi đã giải phóng (use-after-free) (C6.4)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>memory</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>REQ-17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>H6: Mã PIN két thủ kho lưu tạm trong bộ nhớ phải được xóa sạch (zero-out) trước khi free (C6.5)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>security</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>REQ-05</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>H5: Ghi nhật ký chuẩn hóa với printf("%s") và không rò rỉ RAM</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>safety</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>REQ-06</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>H6: Đồng bộ hóa phiên kho bằng Mutex và xóa dữ liệu nhạy cảm trước khi giải phóng</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>concurrency</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>REQ-18</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Toàn bộ luồng phiếu kho: Luôn kết thúc hợp lệ và tồn tại nhánh từ chối đầu vào độc hại</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>liveness</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -634,630 +973,416 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TrangThai</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>KhoiTao</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Nhan</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>ChuyenDenCacTrangThai</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>MaTruongHop</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>GhiChu</t>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>DichChuyenDen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>start</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>start, safe</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>h1_vao</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Bắt đầu xử lý phiếu kho</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>h1_vao</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>h1, receiving</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>h1_ok, h1_tu_choi</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Nhận chuỗi mã phiếu</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>h1_ok</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>h1, input_ok, safe</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>h2_vao</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>C1.1</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Mã phiếu hợp lệ</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>h1_tu_choi</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>h1, input_rejected, safe</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>ket_thuc_tu_choi</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>C1.2</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Từ chối chuỗi quá dài an toàn</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>h2_vao</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>h2, allocating</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>h2_ok, h2_tu_choi</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>H2</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Cấp phát danh mục heap</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>h2_ok</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>h2, allocated, initialized, safe</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>h3_vao</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>C2.1</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Cấp phát và dọn dẹp an toàn</t>
-        </is>
-      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>h2_tu_choi</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>h2, input_rejected, safe</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>ket_thuc_tu_choi</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>C2.2</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Báo lỗi RAM và dọn dẹp sạch sẽ</t>
-        </is>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>h3_vao</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>h3, computing</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>h3_ok, h3_tu_choi</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>H3</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Tính toán tồn kho an toàn</t>
-        </is>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>h3_ok</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>h3, amount_ok, safe</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>h4_vao</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>C3.1</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Tính toán chuẩn xác</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>h3_tu_choi</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>h3, input_rejected, safe</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>ket_thuc_tu_choi</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>C3.2</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Phát hiện nguy cơ tràn số, từ chối an toàn</t>
-        </is>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>h4_vao</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>h4, token_received</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>h4_ok, h4_tu_choi</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>H4</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Xác thực token thủ kho</t>
-        </is>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>h4_ok</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>h4, token_verified, safe</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>h5_vao</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>C4.1</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Xác thực hợp lệ</t>
-        </is>
-      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>h4_tu_choi</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>h4, input_rejected, safe</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>ket_thuc_tu_choi</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>C4.2</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Từ chối token sai quy cách</t>
-        </is>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>h5_vao</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>h5, logging</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>h5_ok</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>H5</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Ghi nhật ký kiểm kê an toàn</t>
-        </is>
-      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>h5_ok</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>h5, log_freed, safe</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>h6_phien_ranh</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>C5.1</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Ghi log an toàn</t>
-        </is>
-      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>h6_phien_ranh</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>h6, sess_free</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>h6_nhap_giu, h6_xuat_giu</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>H6</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Phiên kho ở trạng thái rảnh</t>
-        </is>
-      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>h6_nhap_giu</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>h6, nhap_locked</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>h6_giai_phong</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>C6.1</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Khóa mutex phiên kho</t>
-        </is>
-      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>h6_xuat_giu</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>h6, xuat_locked</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>h6_giai_phong</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>C6.1</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Khóa mutex phiên kho</t>
-        </is>
-      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>h6_giai_phong</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>h6, releasing</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>ket_thuc_ok</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>C6.1</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Dọn dẹp và xóa mã PIN két kho</t>
-        </is>
-      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>ket_thuc_ok</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>flow_end, stock_done, mem_clean, safe</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>ket_thuc_ok</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Hoàn tất an toàn</t>
-        </is>
-      </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>ket_thuc_tu_choi</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>flow_end, input_rejected, mem_clean, safe</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>ket_thuc_tu_choi</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Từ chối an toàn</t>
         </is>
       </c>
     </row>
@@ -1272,234 +1397,402 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>CongThucCTL</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>GhiChu</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ynghia</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>KetQuaKiemChung</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>AG(!violation)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Safety tổng quát: Luôn thỏa mãn</t>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Không bao giờ rơi vào bất kỳ trạng thái vi phạm an toàn nào</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>AG(!buffer_overflow)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Safety: Không bao giờ tràn bộ đệm</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>H1: Không bao giờ tràn bộ đệm stack (CWE-121)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>AG(!off_by_one)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Safety: Không bao giờ tràn 1 byte</t>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>H1: Không bao giờ ghi đè byte ranh giới bộ đệm (CWE-193)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>AG(!null_deref)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Safety: Không bao giờ null dereference</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>H2: Không bao giờ giải tham chiếu con trỏ NULL sau malloc (CWE-476)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>AG(!alloc_size_overflow)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Safety: Không tràn kích thước heap</t>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>H2: Không bao giờ tính sai kích thước cấp phát heap</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>AG(!uninit_read)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Safety: Không đọc bộ nhớ rác</t>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>H2: Không bao giờ đọc dữ liệu rác trước khi khởi tạo (CWE-457)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>AG(!int_overflow)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Safety: Không tràn số nguyên</t>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>H3: Không bao giờ tràn số nguyên có dấu khi cộng dồn tồn kho (CWE-190)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>AG(!negative_amount)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Safety: Không có số tiền âm</t>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>H3: Không bao giờ chấp nhận số lượng nhập hàng là số âm</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>AG(!div_by_zero)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Safety: Không chia cho 0</t>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>H3: Không bao giờ chia cho 0 khi tính đơn giá bình quân (CWE-369)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>AG(!hidden_bypass)</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Safety: Không có cửa sau backdoor</t>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>H4: Không có nhánh ẩn bypass xác thực quyền thủ kho (CWE-285)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>AG(!mem_leak)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Safety: 0 byte rò rỉ bộ nhớ</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>H5: Không bị rò rỉ bộ nhớ log khi thoát sớm (CWE-401)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>AG(!format_string)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Safety: Không có lỗi format string</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>H5: Không đưa chuỗi người dùng vào định dạng printf (CWE-134)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>AG(!race)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Safety: Không có tranh chấp khóa</t>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>H6: Không có tranh chấp phiên kho giữa 2 tiến trình (CWE-667)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>AG(!double_free)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Safety: Không bao giờ double free</t>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>H6: Không bao giờ giải phóng bộ nhớ 2 lần (CWE-415)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>AG(!use_after_free)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Safety: Không bao giờ use-after-free</t>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>H6: Không bao giờ đọc con trỏ sau khi free (CWE-416)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>AG(!secret_residue)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Safety: Xóa sạch mã PIN trước khi free</t>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>H6: Không để sót mã PIN két kho trong RAM sau khi đóng phiên (CWE-226)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>AF(flow_end)</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Liveness: Luôn hoàn tất</t>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Mọi đường đi thực thi đều kết thúc hợp lệ, không deadlock</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>EF(stock_done)</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Reachability: Tồn tại đường đi thành công</t>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Tồn tại kịch bản nhập kho thành công trọn vẹn</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>EF(input_rejected)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Tồn tại kịch bản từ chối đầu vào độc hại bảo vệ hệ thống</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>EG(!violation)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Tồn tại ít nhất một đường đi hoàn toàn an toàn</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>EF(nhap_locked)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Tiến trình nhập kho có thể chiếm giữ khóa phiên</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>EF(xuat_locked)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Tiến trình xuất kho có thể chiếm giữ khóa phiên</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>THỎA MÃN (ĐÚNG - ĐÃ ĐƯỢC VÁ AN TOÀN)</t>
         </is>
       </c>
     </row>

</xml_diff>